<commit_message>
Show South Africa archive dates as dd-mmm-yyyy
pandas' default "YYYY-MM-DD" in a narrow column was displayed by some
viewers as "26/9" (year and month only), so every September row looked
the same date. The date column is now written as e.g. 15-Sep-2026 with a
wider column - only in this script, not in the shared xlsx_notes helper.
Existing archive reformatted in place; reading it back is unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VTzJJ2guyTYFmhjpVDkmA1
</commit_message>
<xml_diff>
--- a/south_africa/south_africa_generation_mix_daily.xlsx
+++ b/south_africa/south_africa_generation_mix_daily.xlsx
@@ -18,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="dd-mmm-yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -59,9 +59,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -455,9 +456,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr"/>
-    </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -479,9 +478,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
@@ -496,9 +493,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
@@ -526,6 +521,9 @@
   </sheetPr>
   <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -580,7 +578,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
+      <c r="A2" s="3" t="n">
         <v>46280</v>
       </c>
       <c r="B2" t="n">
@@ -612,7 +610,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>46281</v>
       </c>
       <c r="B3" t="n">
@@ -644,7 +642,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>46282</v>
       </c>
       <c r="B4" t="n">
@@ -676,7 +674,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>46283</v>
       </c>
       <c r="B5" t="n">
@@ -708,7 +706,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>46284</v>
       </c>
       <c r="B6" t="n">
@@ -740,7 +738,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n">
+      <c r="A7" s="3" t="n">
         <v>46285</v>
       </c>
       <c r="B7" t="n">
@@ -772,7 +770,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n">
+      <c r="A8" s="3" t="n">
         <v>46286</v>
       </c>
       <c r="B8" t="n">
@@ -804,7 +802,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n">
+      <c r="A9" s="3" t="n">
         <v>46287</v>
       </c>
       <c r="B9" t="n">
@@ -836,7 +834,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n">
+      <c r="A10" s="3" t="n">
         <v>46288</v>
       </c>
       <c r="B10" t="n">
@@ -868,7 +866,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n">
+      <c r="A11" s="3" t="n">
         <v>46289</v>
       </c>
       <c r="B11" t="n">

</xml_diff>